<commit_message>
[update] bullit 레벨업 가능함
최대 레벨 도달 시 게임이 터져버림. 아마 반복문안에 무한 루프가 도는것으로 예상이 됨.
최대 레벨 도달 관련 메서드 원인분석 필요함
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/WJBullitLv.xlsx
+++ b/JsonConverter/ExcelFiles/WJBullitLv.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\OZ_Project\WJMainProject2D\JsonConverter\ExcelFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3474EE94-FAE1-4BDC-A7E0-C51E30D7E3F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08195AFA-7F2C-49E7-A0DB-62C956C0C2A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10680" yWindow="3375" windowWidth="17115" windowHeight="11145" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="420" yWindow="375" windowWidth="17115" windowHeight="11145" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="WJTable_Bullit" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="29">
   <si>
     <t>(name)</t>
   </si>
@@ -105,22 +105,6 @@
   </si>
   <si>
     <t>Basic</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>Double</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>Triple</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>DoubleFiring</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>TripleFiring</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
@@ -527,7 +511,7 @@
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="15.75" customHeight="1">
@@ -573,7 +557,7 @@
         <v>20</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="15.75" customHeight="1">
@@ -596,7 +580,7 @@
         <v>21</v>
       </c>
       <c r="G4" s="12" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="H4" s="3"/>
       <c r="I4" s="3"/>
@@ -619,10 +603,10 @@
         <v>13</v>
       </c>
       <c r="F5" s="12" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G5" s="12" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
@@ -645,10 +629,10 @@
         <v>13</v>
       </c>
       <c r="F6" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="G6" s="12" t="s">
         <v>23</v>
-      </c>
-      <c r="G6" s="12" t="s">
-        <v>27</v>
       </c>
       <c r="H6" s="3"/>
       <c r="I6" s="3"/>
@@ -670,11 +654,11 @@
       <c r="E7" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="F7" s="12" t="s">
         <v>21</v>
       </c>
       <c r="G7" s="12" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="H7" s="3"/>
       <c r="I7" s="3"/>
@@ -696,11 +680,11 @@
       <c r="E8" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="F8" s="6" t="s">
-        <v>24</v>
+      <c r="F8" s="12" t="s">
+        <v>21</v>
       </c>
       <c r="G8" s="12" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="H8" s="3"/>
       <c r="I8" s="3"/>
@@ -722,11 +706,11 @@
       <c r="E9" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="F9" s="6" t="s">
-        <v>25</v>
+      <c r="F9" s="12" t="s">
+        <v>21</v>
       </c>
       <c r="G9" s="12" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="H9" s="3"/>
       <c r="I9" s="3"/>
@@ -734,7 +718,7 @@
     </row>
     <row r="10" spans="1:10" ht="15.75" customHeight="1">
       <c r="A10" s="7" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B10" s="7">
         <v>5</v>
@@ -746,13 +730,13 @@
         <v>2</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="F10" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="F10" s="12" t="s">
         <v>21</v>
       </c>
       <c r="G10" s="12" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="H10" s="3"/>
       <c r="I10" s="3"/>
@@ -760,7 +744,7 @@
     </row>
     <row r="11" spans="1:10" ht="15.75" customHeight="1">
       <c r="A11" s="7" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B11" s="7">
         <v>10</v>
@@ -772,13 +756,13 @@
         <v>1</v>
       </c>
       <c r="E11" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="F11" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="F11" s="12" t="s">
         <v>21</v>
       </c>
       <c r="G11" s="12" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="H11" s="3"/>
       <c r="I11" s="3"/>
@@ -786,7 +770,7 @@
     </row>
     <row r="12" spans="1:10" ht="15.75" customHeight="1">
       <c r="A12" s="7" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="B12" s="6">
         <v>25</v>
@@ -798,13 +782,13 @@
         <v>0.5</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="F12" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="F12" s="12" t="s">
         <v>21</v>
       </c>
       <c r="G12" s="12" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="H12" s="3"/>
       <c r="I12" s="3"/>

</xml_diff>

<commit_message>
[update] Bullit 생산 방식 변화 구현
레벨에 따라 더블 샷, 트리플 샷 구현
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/WJBullitLv.xlsx
+++ b/JsonConverter/ExcelFiles/WJBullitLv.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\OZ_Project\WJMainProject2D\JsonConverter\ExcelFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08195AFA-7F2C-49E7-A0DB-62C956C0C2A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1621F2DD-66F7-419D-A1DC-322B40891A16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="420" yWindow="375" windowWidth="17115" windowHeight="11145" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10875" yWindow="855" windowWidth="17115" windowHeight="11145" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="WJTable_Bullit" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="31">
   <si>
     <t>(name)</t>
   </si>
@@ -131,6 +131,14 @@
   </si>
   <si>
     <t>2D/WJ_Folder/Sprite/Arrow</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>DoubleFiring</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>TripleFiring</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
@@ -681,7 +689,7 @@
         <v>12</v>
       </c>
       <c r="F8" s="12" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="G8" s="12" t="s">
         <v>23</v>
@@ -707,7 +715,7 @@
         <v>12</v>
       </c>
       <c r="F9" s="12" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="G9" s="12" t="s">
         <v>23</v>

</xml_diff>

<commit_message>
[update] MeleeAtk 구현 완료
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/WJBullitLv.xlsx
+++ b/JsonConverter/ExcelFiles/WJBullitLv.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\OZ_Project\WJMainProject2D\JsonConverter\ExcelFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC85C6BA-FE10-4F0D-A11A-472D70593A04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F58F76C-BD68-4AD5-BD38-A0DE79A6D90A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6420" yWindow="2115" windowWidth="18780" windowHeight="11145" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2775" yWindow="1590" windowWidth="22485" windowHeight="11145" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="WJTable_Bullit" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="46">
   <si>
     <t>(name)</t>
   </si>
@@ -183,6 +183,18 @@
   </si>
   <si>
     <t>150</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>_animatorPath</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>MeleeDoubleSize</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>MeleeTripleSize</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
@@ -939,6 +951,7 @@
     <col min="6" max="6" width="18.28515625" customWidth="1"/>
     <col min="7" max="7" width="23.7109375" customWidth="1"/>
     <col min="8" max="8" width="15.85546875" customWidth="1"/>
+    <col min="9" max="9" width="31.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="69.75" customHeight="1">
@@ -956,6 +969,7 @@
         <v>22</v>
       </c>
       <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
     </row>
     <row r="2" spans="1:10" ht="15.75" customHeight="1">
       <c r="A2" s="1" t="s">
@@ -982,6 +996,9 @@
       <c r="H2" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="I2" s="1" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="3" spans="1:10" ht="15.75" customHeight="1" thickBot="1">
       <c r="A3" s="24" t="s">
@@ -1008,6 +1025,9 @@
       <c r="H3" s="24" t="s">
         <v>41</v>
       </c>
+      <c r="I3" s="24" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="4" spans="1:10" ht="15.75" customHeight="1" thickBot="1">
       <c r="A4" s="25" t="s">
@@ -1034,7 +1054,7 @@
       <c r="H4" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="I4" s="2"/>
+      <c r="I4" s="13"/>
       <c r="J4" s="2"/>
     </row>
     <row r="5" spans="1:10" ht="15.75" customHeight="1" thickBot="1">
@@ -1062,7 +1082,7 @@
       <c r="H5" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="I5" s="2"/>
+      <c r="I5" s="9"/>
       <c r="J5" s="2"/>
     </row>
     <row r="6" spans="1:10" ht="15.75" customHeight="1" thickBot="1">
@@ -1090,7 +1110,7 @@
       <c r="H6" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="I6" s="2"/>
+      <c r="I6" s="18"/>
       <c r="J6" s="2"/>
     </row>
     <row r="7" spans="1:10" ht="15.75" customHeight="1" thickBot="1">
@@ -1118,7 +1138,7 @@
       <c r="H7" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="I7" s="2"/>
+      <c r="I7" s="13"/>
       <c r="J7" s="2"/>
     </row>
     <row r="8" spans="1:10" ht="15.75" customHeight="1" thickBot="1">
@@ -1146,7 +1166,7 @@
       <c r="H8" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="I8" s="2"/>
+      <c r="I8" s="9"/>
       <c r="J8" s="2"/>
     </row>
     <row r="9" spans="1:10" ht="15.75" customHeight="1" thickBot="1">
@@ -1174,7 +1194,7 @@
       <c r="H9" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="I9" s="2"/>
+      <c r="I9" s="18"/>
       <c r="J9" s="2"/>
     </row>
     <row r="10" spans="1:10" ht="15.75" customHeight="1" thickBot="1">
@@ -1202,7 +1222,7 @@
       <c r="H10" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="I10" s="2"/>
+      <c r="I10" s="13"/>
       <c r="J10" s="2"/>
     </row>
     <row r="11" spans="1:10" ht="15.75" customHeight="1" thickBot="1">
@@ -1230,7 +1250,7 @@
       <c r="H11" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="I11" s="2"/>
+      <c r="I11" s="9"/>
       <c r="J11" s="2"/>
     </row>
     <row r="12" spans="1:10" ht="15.75" customHeight="1" thickBot="1">
@@ -1258,7 +1278,7 @@
       <c r="H12" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="I12" s="2"/>
+      <c r="I12" s="41"/>
       <c r="J12" s="2"/>
     </row>
     <row r="13" spans="1:10" ht="15.75" customHeight="1" thickBot="1">
@@ -1286,7 +1306,9 @@
       <c r="H13" s="21">
         <v>10</v>
       </c>
-      <c r="I13" s="2"/>
+      <c r="I13" s="21" t="s">
+        <v>38</v>
+      </c>
       <c r="J13" s="2"/>
     </row>
     <row r="14" spans="1:10" ht="15.75" customHeight="1" thickBot="1">
@@ -1306,7 +1328,7 @@
         <v>38</v>
       </c>
       <c r="F14" s="36" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="G14" s="43" t="s">
         <v>40</v>
@@ -1314,7 +1336,9 @@
       <c r="H14" s="21">
         <v>10</v>
       </c>
-      <c r="I14" s="2"/>
+      <c r="I14" s="10" t="s">
+        <v>38</v>
+      </c>
       <c r="J14" s="2"/>
     </row>
     <row r="15" spans="1:10" ht="15.75" customHeight="1" thickBot="1">
@@ -1334,7 +1358,7 @@
         <v>38</v>
       </c>
       <c r="F15" s="37" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="G15" s="44" t="s">
         <v>40</v>
@@ -1342,7 +1366,9 @@
       <c r="H15" s="21">
         <v>10</v>
       </c>
-      <c r="I15" s="2"/>
+      <c r="I15" s="34" t="s">
+        <v>38</v>
+      </c>
       <c r="J15" s="2"/>
     </row>
     <row r="16" spans="1:10" ht="15.75" customHeight="1">
@@ -1354,8 +1380,9 @@
       <c r="F16" s="30"/>
       <c r="G16" s="30"/>
       <c r="H16" s="30"/>
-    </row>
-    <row r="17" spans="1:8" ht="15.75" customHeight="1">
+      <c r="I16" s="30"/>
+    </row>
+    <row r="17" spans="1:9" ht="15.75" customHeight="1">
       <c r="A17" s="6"/>
       <c r="B17" s="6"/>
       <c r="C17" s="6"/>
@@ -1364,8 +1391,9 @@
       <c r="F17" s="6"/>
       <c r="G17" s="6"/>
       <c r="H17" s="6"/>
-    </row>
-    <row r="18" spans="1:8" ht="15.75" customHeight="1">
+      <c r="I17" s="6"/>
+    </row>
+    <row r="18" spans="1:9" ht="15.75" customHeight="1">
       <c r="A18" s="6"/>
       <c r="B18" s="6"/>
       <c r="C18" s="6"/>
@@ -1374,8 +1402,9 @@
       <c r="F18" s="6"/>
       <c r="G18" s="6"/>
       <c r="H18" s="6"/>
-    </row>
-    <row r="19" spans="1:8" ht="15.75" customHeight="1">
+      <c r="I18" s="6"/>
+    </row>
+    <row r="19" spans="1:9" ht="15.75" customHeight="1">
       <c r="A19" s="6"/>
       <c r="B19" s="6"/>
       <c r="C19" s="6"/>
@@ -1384,8 +1413,9 @@
       <c r="F19" s="6"/>
       <c r="G19" s="6"/>
       <c r="H19" s="6"/>
-    </row>
-    <row r="20" spans="1:8" ht="15.75" customHeight="1">
+      <c r="I19" s="6"/>
+    </row>
+    <row r="20" spans="1:9" ht="15.75" customHeight="1">
       <c r="A20" s="6"/>
       <c r="B20" s="6"/>
       <c r="C20" s="6"/>
@@ -1394,8 +1424,9 @@
       <c r="F20" s="6"/>
       <c r="G20" s="6"/>
       <c r="H20" s="6"/>
-    </row>
-    <row r="21" spans="1:8" ht="15.75" customHeight="1">
+      <c r="I20" s="6"/>
+    </row>
+    <row r="21" spans="1:9" ht="15.75" customHeight="1">
       <c r="A21" s="6"/>
       <c r="B21" s="6"/>
       <c r="C21" s="6"/>
@@ -1404,8 +1435,9 @@
       <c r="F21" s="6"/>
       <c r="G21" s="6"/>
       <c r="H21" s="6"/>
-    </row>
-    <row r="22" spans="1:8" ht="15.75" customHeight="1">
+      <c r="I21" s="6"/>
+    </row>
+    <row r="22" spans="1:9" ht="15.75" customHeight="1">
       <c r="A22" s="6"/>
       <c r="B22" s="6"/>
       <c r="C22" s="6"/>
@@ -1414,8 +1446,9 @@
       <c r="F22" s="6"/>
       <c r="G22" s="6"/>
       <c r="H22" s="6"/>
-    </row>
-    <row r="23" spans="1:8" ht="15.75" customHeight="1">
+      <c r="I22" s="6"/>
+    </row>
+    <row r="23" spans="1:9" ht="15.75" customHeight="1">
       <c r="A23" s="6"/>
       <c r="B23" s="6"/>
       <c r="C23" s="6"/>
@@ -1424,8 +1457,9 @@
       <c r="F23" s="6"/>
       <c r="G23" s="6"/>
       <c r="H23" s="6"/>
-    </row>
-    <row r="24" spans="1:8" ht="15.75" customHeight="1">
+      <c r="I23" s="6"/>
+    </row>
+    <row r="24" spans="1:9" ht="15.75" customHeight="1">
       <c r="A24" s="6"/>
       <c r="B24" s="6"/>
       <c r="C24" s="6"/>
@@ -1434,8 +1468,9 @@
       <c r="F24" s="6"/>
       <c r="G24" s="6"/>
       <c r="H24" s="6"/>
-    </row>
-    <row r="25" spans="1:8" ht="15.75" customHeight="1">
+      <c r="I24" s="6"/>
+    </row>
+    <row r="25" spans="1:9" ht="15.75" customHeight="1">
       <c r="A25" s="6"/>
       <c r="B25" s="6"/>
       <c r="C25" s="6"/>
@@ -1444,8 +1479,9 @@
       <c r="F25" s="6"/>
       <c r="G25" s="6"/>
       <c r="H25" s="6"/>
-    </row>
-    <row r="26" spans="1:8" ht="15.75" customHeight="1">
+      <c r="I25" s="6"/>
+    </row>
+    <row r="26" spans="1:9" ht="15.75" customHeight="1">
       <c r="A26" s="7"/>
       <c r="B26" s="7"/>
       <c r="C26" s="7"/>
@@ -1454,8 +1490,9 @@
       <c r="F26" s="7"/>
       <c r="G26" s="7"/>
       <c r="H26" s="7"/>
-    </row>
-    <row r="27" spans="1:8" ht="15.75" customHeight="1">
+      <c r="I26" s="7"/>
+    </row>
+    <row r="27" spans="1:9" ht="15.75" customHeight="1">
       <c r="A27" s="7"/>
       <c r="B27" s="7"/>
       <c r="C27" s="7"/>
@@ -1464,8 +1501,9 @@
       <c r="F27" s="7"/>
       <c r="G27" s="7"/>
       <c r="H27" s="7"/>
-    </row>
-    <row r="28" spans="1:8" ht="15.75" customHeight="1">
+      <c r="I27" s="7"/>
+    </row>
+    <row r="28" spans="1:9" ht="15.75" customHeight="1">
       <c r="A28" s="7"/>
       <c r="B28" s="7"/>
       <c r="C28" s="7"/>
@@ -1474,8 +1512,9 @@
       <c r="F28" s="7"/>
       <c r="G28" s="7"/>
       <c r="H28" s="7"/>
-    </row>
-    <row r="29" spans="1:8" ht="15.75" customHeight="1">
+      <c r="I28" s="7"/>
+    </row>
+    <row r="29" spans="1:9" ht="15.75" customHeight="1">
       <c r="A29" s="7"/>
       <c r="B29" s="7"/>
       <c r="C29" s="7"/>
@@ -1484,8 +1523,9 @@
       <c r="F29" s="7"/>
       <c r="G29" s="7"/>
       <c r="H29" s="7"/>
-    </row>
-    <row r="30" spans="1:8" ht="15.75" customHeight="1">
+      <c r="I29" s="7"/>
+    </row>
+    <row r="30" spans="1:9" ht="15.75" customHeight="1">
       <c r="A30" s="7"/>
       <c r="B30" s="7"/>
       <c r="C30" s="7"/>
@@ -1494,8 +1534,9 @@
       <c r="F30" s="7"/>
       <c r="G30" s="7"/>
       <c r="H30" s="7"/>
-    </row>
-    <row r="31" spans="1:8" ht="15.75" customHeight="1">
+      <c r="I30" s="7"/>
+    </row>
+    <row r="31" spans="1:9" ht="15.75" customHeight="1">
       <c r="A31" s="7"/>
       <c r="B31" s="7"/>
       <c r="C31" s="7"/>
@@ -1504,8 +1545,9 @@
       <c r="F31" s="7"/>
       <c r="G31" s="7"/>
       <c r="H31" s="7"/>
-    </row>
-    <row r="32" spans="1:8" ht="15.75" customHeight="1">
+      <c r="I31" s="7"/>
+    </row>
+    <row r="32" spans="1:9" ht="15.75" customHeight="1">
       <c r="A32" s="8"/>
       <c r="B32" s="8"/>
       <c r="C32" s="8"/>
@@ -1514,8 +1556,9 @@
       <c r="F32" s="8"/>
       <c r="G32" s="8"/>
       <c r="H32" s="8"/>
-    </row>
-    <row r="33" spans="1:8" ht="15.75" customHeight="1">
+      <c r="I32" s="8"/>
+    </row>
+    <row r="33" spans="1:9" ht="15.75" customHeight="1">
       <c r="A33" s="8"/>
       <c r="B33" s="8"/>
       <c r="C33" s="8"/>
@@ -1524,8 +1567,9 @@
       <c r="F33" s="8"/>
       <c r="G33" s="8"/>
       <c r="H33" s="8"/>
-    </row>
-    <row r="34" spans="1:8" ht="15.75" customHeight="1">
+      <c r="I33" s="8"/>
+    </row>
+    <row r="34" spans="1:9" ht="15.75" customHeight="1">
       <c r="A34" s="8"/>
       <c r="B34" s="8"/>
       <c r="C34" s="8"/>
@@ -1534,8 +1578,9 @@
       <c r="F34" s="8"/>
       <c r="G34" s="8"/>
       <c r="H34" s="8"/>
-    </row>
-    <row r="35" spans="1:8" ht="15.75" customHeight="1">
+      <c r="I34" s="8"/>
+    </row>
+    <row r="35" spans="1:9" ht="15.75" customHeight="1">
       <c r="A35" s="8"/>
       <c r="B35" s="8"/>
       <c r="C35" s="8"/>
@@ -1544,20 +1589,21 @@
       <c r="F35" s="8"/>
       <c r="G35" s="8"/>
       <c r="H35" s="8"/>
-    </row>
-    <row r="36" spans="1:8" ht="15.75" customHeight="1"/>
-    <row r="37" spans="1:8" ht="15.75" customHeight="1"/>
-    <row r="38" spans="1:8" ht="15.75" customHeight="1"/>
-    <row r="39" spans="1:8" ht="15.75" customHeight="1"/>
-    <row r="40" spans="1:8" ht="15.75" customHeight="1"/>
-    <row r="41" spans="1:8" ht="15.75" customHeight="1"/>
-    <row r="42" spans="1:8" ht="15.75" customHeight="1"/>
-    <row r="43" spans="1:8" ht="15.75" customHeight="1"/>
-    <row r="44" spans="1:8" ht="15.75" customHeight="1"/>
-    <row r="45" spans="1:8" ht="15.75" customHeight="1"/>
-    <row r="46" spans="1:8" ht="15.75" customHeight="1"/>
-    <row r="47" spans="1:8" ht="15.75" customHeight="1"/>
-    <row r="48" spans="1:8" ht="15.75" customHeight="1"/>
+      <c r="I35" s="8"/>
+    </row>
+    <row r="36" spans="1:9" ht="15.75" customHeight="1"/>
+    <row r="37" spans="1:9" ht="15.75" customHeight="1"/>
+    <row r="38" spans="1:9" ht="15.75" customHeight="1"/>
+    <row r="39" spans="1:9" ht="15.75" customHeight="1"/>
+    <row r="40" spans="1:9" ht="15.75" customHeight="1"/>
+    <row r="41" spans="1:9" ht="15.75" customHeight="1"/>
+    <row r="42" spans="1:9" ht="15.75" customHeight="1"/>
+    <row r="43" spans="1:9" ht="15.75" customHeight="1"/>
+    <row r="44" spans="1:9" ht="15.75" customHeight="1"/>
+    <row r="45" spans="1:9" ht="15.75" customHeight="1"/>
+    <row r="46" spans="1:9" ht="15.75" customHeight="1"/>
+    <row r="47" spans="1:9" ht="15.75" customHeight="1"/>
+    <row r="48" spans="1:9" ht="15.75" customHeight="1"/>
     <row r="49" ht="15.75" customHeight="1"/>
     <row r="50" ht="15.75" customHeight="1"/>
     <row r="51" ht="15.75" customHeight="1"/>

</xml_diff>